<commit_message>
Upgrade intensive engine with Bangbet, Soccabet, Supabet scrapers & market pairings
</commit_message>
<xml_diff>
--- a/football/data/quasi_arb_ml.xlsx
+++ b/football/data/quasi_arb_ml.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q202"/>
+  <dimension ref="A1:Q204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12612,10 +12612,8 @@
           <t>Over/Under</t>
         </is>
       </c>
-      <c r="H199" t="inlineStr">
-        <is>
-          <t>3.5</t>
-        </is>
+      <c r="H199" t="n">
+        <v>3.5</v>
       </c>
       <c r="I199" t="inlineStr">
         <is>
@@ -12677,10 +12675,8 @@
           <t>Over/Under</t>
         </is>
       </c>
-      <c r="H200" t="inlineStr">
-        <is>
-          <t>3.5</t>
-        </is>
+      <c r="H200" t="n">
+        <v>3.5</v>
       </c>
       <c r="I200" t="inlineStr">
         <is>
@@ -12742,10 +12738,8 @@
           <t>Over/Under</t>
         </is>
       </c>
-      <c r="H201" t="inlineStr">
-        <is>
-          <t>3.5</t>
-        </is>
+      <c r="H201" t="n">
+        <v>3.5</v>
       </c>
       <c r="I201" t="inlineStr">
         <is>
@@ -12807,10 +12801,8 @@
           <t>Over/Under</t>
         </is>
       </c>
-      <c r="H202" t="inlineStr">
-        <is>
-          <t>3.5</t>
-        </is>
+      <c r="H202" t="n">
+        <v>3.5</v>
       </c>
       <c r="I202" t="inlineStr">
         <is>
@@ -12836,6 +12828,136 @@
       <c r="P202" t="inlineStr"/>
       <c r="Q202" t="inlineStr"/>
     </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-06-17 22:47:28</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Asian Over/Under</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>U2.0</t>
+        </is>
+      </c>
+      <c r="J203" t="n">
+        <v>2.5744</v>
+      </c>
+      <c r="K203" t="n">
+        <v>11.07</v>
+      </c>
+      <c r="L203" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>1xBet, Sportybet</t>
+        </is>
+      </c>
+      <c r="N203" t="inlineStr"/>
+      <c r="O203" t="inlineStr"/>
+      <c r="P203" t="inlineStr"/>
+      <c r="Q203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-06-17 22:47:28</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>Asian Over/Under</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>U2.0</t>
+        </is>
+      </c>
+      <c r="J204" t="n">
+        <v>3.9116</v>
+      </c>
+      <c r="K204" t="n">
+        <v>16.82</v>
+      </c>
+      <c r="L204" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>1xBet, 22Bet</t>
+        </is>
+      </c>
+      <c r="N204" t="inlineStr"/>
+      <c r="O204" t="inlineStr"/>
+      <c r="P204" t="inlineStr"/>
+      <c r="Q204" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Optimize Soccabet scraper to be ultra-fast and fetch all today matches
</commit_message>
<xml_diff>
--- a/football/data/quasi_arb_ml.xlsx
+++ b/football/data/quasi_arb_ml.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q212"/>
+  <dimension ref="A1:Q258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13431,10 +13431,8 @@
           <t>Bookings Over/Under</t>
         </is>
       </c>
-      <c r="H212" t="inlineStr">
-        <is>
-          <t>3.5</t>
-        </is>
+      <c r="H212" t="n">
+        <v>3.5</v>
       </c>
       <c r="I212" t="inlineStr">
         <is>
@@ -13460,6 +13458,2834 @@
       <c r="P212" t="inlineStr"/>
       <c r="Q212" t="inlineStr"/>
     </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:22:52</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr"/>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="J213" t="n">
+        <v>0.2419</v>
+      </c>
+      <c r="K213" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="L213" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>1xBet, Sportybet, Soccabet</t>
+        </is>
+      </c>
+      <c r="N213" t="inlineStr"/>
+      <c r="O213" t="inlineStr"/>
+      <c r="P213" t="inlineStr"/>
+      <c r="Q213" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:22:52</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr"/>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="J214" t="n">
+        <v>1.7209</v>
+      </c>
+      <c r="K214" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="L214" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>1xBet, Soccabet, Soccabet</t>
+        </is>
+      </c>
+      <c r="N214" t="inlineStr"/>
+      <c r="O214" t="inlineStr"/>
+      <c r="P214" t="inlineStr"/>
+      <c r="Q214" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:22:52</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>CA Quilmes Reserve</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>San Martin de San Juan Reserve</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Primera LPF, Reserves</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="H215" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>U2.5</t>
+        </is>
+      </c>
+      <c r="J215" t="n">
+        <v>62.1628</v>
+      </c>
+      <c r="K215" t="n">
+        <v>267.3</v>
+      </c>
+      <c r="L215" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>Sportybet, Betway</t>
+        </is>
+      </c>
+      <c r="N215" t="inlineStr"/>
+      <c r="O215" t="inlineStr"/>
+      <c r="P215" t="inlineStr"/>
+      <c r="Q215" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:22:52</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>CA Quilmes Reserve</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>San Martin de San Juan Reserve</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Primera LPF, Reserves</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="H216" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>U2.5</t>
+        </is>
+      </c>
+      <c r="J216" t="n">
+        <v>68.64879999999999</v>
+      </c>
+      <c r="K216" t="n">
+        <v>295.19</v>
+      </c>
+      <c r="L216" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>Sportybet, MSport</t>
+        </is>
+      </c>
+      <c r="N216" t="inlineStr"/>
+      <c r="O216" t="inlineStr"/>
+      <c r="P216" t="inlineStr"/>
+      <c r="Q216" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:22:52</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>CA Quilmes Reserve</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>San Martin de San Juan Reserve</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Primera LPF, Reserves</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="H217" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>U2.5</t>
+        </is>
+      </c>
+      <c r="J217" t="n">
+        <v>49.1907</v>
+      </c>
+      <c r="K217" t="n">
+        <v>211.52</v>
+      </c>
+      <c r="L217" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>Sportybet, Bangbet</t>
+        </is>
+      </c>
+      <c r="N217" t="inlineStr"/>
+      <c r="O217" t="inlineStr"/>
+      <c r="P217" t="inlineStr"/>
+      <c r="Q217" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:22:52</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>CA Quilmes Reserve</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>San Martin de San Juan Reserve</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Primera LPF, Reserves</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="H218" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>U2.5</t>
+        </is>
+      </c>
+      <c r="J218" t="n">
+        <v>42.7023</v>
+      </c>
+      <c r="K218" t="n">
+        <v>183.62</v>
+      </c>
+      <c r="L218" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>Sportybet, Supabet</t>
+        </is>
+      </c>
+      <c r="N218" t="inlineStr"/>
+      <c r="O218" t="inlineStr"/>
+      <c r="P218" t="inlineStr"/>
+      <c r="Q218" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:22:52</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>CA Quilmes Reserve</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>San Martin de San Juan Reserve</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Primera LPF, Reserves</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="H219" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>U2.5</t>
+        </is>
+      </c>
+      <c r="J219" t="n">
+        <v>59.8605</v>
+      </c>
+      <c r="K219" t="n">
+        <v>257.4</v>
+      </c>
+      <c r="L219" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>Football.com, Betway</t>
+        </is>
+      </c>
+      <c r="N219" t="inlineStr"/>
+      <c r="O219" t="inlineStr"/>
+      <c r="P219" t="inlineStr"/>
+      <c r="Q219" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:22:52</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>CA Quilmes Reserve</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>San Martin de San Juan Reserve</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Primera LPF, Reserves</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="H220" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>U2.5</t>
+        </is>
+      </c>
+      <c r="J220" t="n">
+        <v>66.25579999999999</v>
+      </c>
+      <c r="K220" t="n">
+        <v>284.9</v>
+      </c>
+      <c r="L220" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>Football.com, MSport</t>
+        </is>
+      </c>
+      <c r="N220" t="inlineStr"/>
+      <c r="O220" t="inlineStr"/>
+      <c r="P220" t="inlineStr"/>
+      <c r="Q220" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:22:52</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>CA Quilmes Reserve</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>San Martin de San Juan Reserve</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Primera LPF, Reserves</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="H221" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>U2.5</t>
+        </is>
+      </c>
+      <c r="J221" t="n">
+        <v>47.0721</v>
+      </c>
+      <c r="K221" t="n">
+        <v>202.41</v>
+      </c>
+      <c r="L221" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>Football.com, Bangbet</t>
+        </is>
+      </c>
+      <c r="N221" t="inlineStr"/>
+      <c r="O221" t="inlineStr"/>
+      <c r="P221" t="inlineStr"/>
+      <c r="Q221" t="inlineStr"/>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:22:52</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>CA Quilmes Reserve</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>San Martin de San Juan Reserve</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>Primera LPF, Reserves</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="H222" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>U2.5</t>
+        </is>
+      </c>
+      <c r="J222" t="n">
+        <v>40.6767</v>
+      </c>
+      <c r="K222" t="n">
+        <v>174.91</v>
+      </c>
+      <c r="L222" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>Football.com, Supabet</t>
+        </is>
+      </c>
+      <c r="N222" t="inlineStr"/>
+      <c r="O222" t="inlineStr"/>
+      <c r="P222" t="inlineStr"/>
+      <c r="Q222" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:22:52</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr"/>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="J223" t="n">
+        <v>1.7535</v>
+      </c>
+      <c r="K223" t="n">
+        <v>7.54</v>
+      </c>
+      <c r="L223" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>Soccabet, Sportybet, Sportybet</t>
+        </is>
+      </c>
+      <c r="N223" t="inlineStr"/>
+      <c r="O223" t="inlineStr"/>
+      <c r="P223" t="inlineStr"/>
+      <c r="Q223" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:22:52</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr"/>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="J224" t="n">
+        <v>1.6279</v>
+      </c>
+      <c r="K224" t="n">
+        <v>7</v>
+      </c>
+      <c r="L224" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>Soccabet, Sportybet, 1xBet</t>
+        </is>
+      </c>
+      <c r="N224" t="inlineStr"/>
+      <c r="O224" t="inlineStr"/>
+      <c r="P224" t="inlineStr"/>
+      <c r="Q224" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:22:52</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr"/>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J225" t="n">
+        <v>1.8791</v>
+      </c>
+      <c r="K225" t="n">
+        <v>8.08</v>
+      </c>
+      <c r="L225" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>Soccabet, Sportybet, 22Bet</t>
+        </is>
+      </c>
+      <c r="N225" t="inlineStr"/>
+      <c r="O225" t="inlineStr"/>
+      <c r="P225" t="inlineStr"/>
+      <c r="Q225" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:22:52</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr"/>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J226" t="n">
+        <v>1.1907</v>
+      </c>
+      <c r="K226" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="L226" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>Soccabet, 22Bet, Sportybet</t>
+        </is>
+      </c>
+      <c r="N226" t="inlineStr"/>
+      <c r="O226" t="inlineStr"/>
+      <c r="P226" t="inlineStr"/>
+      <c r="Q226" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:22:52</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr"/>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="J227" t="n">
+        <v>1.0651</v>
+      </c>
+      <c r="K227" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="L227" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>Soccabet, 22Bet, 1xBet</t>
+        </is>
+      </c>
+      <c r="N227" t="inlineStr"/>
+      <c r="O227" t="inlineStr"/>
+      <c r="P227" t="inlineStr"/>
+      <c r="Q227" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:22:52</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr"/>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J228" t="n">
+        <v>1.3209</v>
+      </c>
+      <c r="K228" t="n">
+        <v>5.68</v>
+      </c>
+      <c r="L228" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>Soccabet, 22Bet, 22Bet</t>
+        </is>
+      </c>
+      <c r="N228" t="inlineStr"/>
+      <c r="O228" t="inlineStr"/>
+      <c r="P228" t="inlineStr"/>
+      <c r="Q228" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:22:52</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>Bookings Over/Under</t>
+        </is>
+      </c>
+      <c r="H229" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>O3.5</t>
+        </is>
+      </c>
+      <c r="J229" t="n">
+        <v>3.3721</v>
+      </c>
+      <c r="K229" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="L229" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>1xBet, Supabet</t>
+        </is>
+      </c>
+      <c r="N229" t="inlineStr"/>
+      <c r="O229" t="inlineStr"/>
+      <c r="P229" t="inlineStr"/>
+      <c r="Q229" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:25:27</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr"/>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J230" t="n">
+        <v>1.8791</v>
+      </c>
+      <c r="K230" t="n">
+        <v>8.08</v>
+      </c>
+      <c r="L230" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>Soccabet, Sportybet, 22Bet</t>
+        </is>
+      </c>
+      <c r="N230" t="inlineStr"/>
+      <c r="O230" t="inlineStr"/>
+      <c r="P230" t="inlineStr"/>
+      <c r="Q230" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:25:27</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr"/>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J231" t="n">
+        <v>1.1907</v>
+      </c>
+      <c r="K231" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="L231" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>Soccabet, 22Bet, Sportybet</t>
+        </is>
+      </c>
+      <c r="N231" t="inlineStr"/>
+      <c r="O231" t="inlineStr"/>
+      <c r="P231" t="inlineStr"/>
+      <c r="Q231" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:28:01</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>CA Quilmes Reserve</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>San Martin de San Juan Reserve</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>Primera LPF, Reserves</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="H232" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>U2.5</t>
+        </is>
+      </c>
+      <c r="J232" t="n">
+        <v>58.9186</v>
+      </c>
+      <c r="K232" t="n">
+        <v>253.35</v>
+      </c>
+      <c r="L232" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>Sportybet, Betway</t>
+        </is>
+      </c>
+      <c r="N232" t="inlineStr"/>
+      <c r="O232" t="inlineStr"/>
+      <c r="P232" t="inlineStr"/>
+      <c r="Q232" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:28:01</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>CA Quilmes Reserve</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>San Martin de San Juan Reserve</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>Primera LPF, Reserves</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>Over/Under</t>
+        </is>
+      </c>
+      <c r="H233" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>U2.5</t>
+        </is>
+      </c>
+      <c r="J233" t="n">
+        <v>56.6628</v>
+      </c>
+      <c r="K233" t="n">
+        <v>243.65</v>
+      </c>
+      <c r="L233" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t>Football.com, Betway</t>
+        </is>
+      </c>
+      <c r="N233" t="inlineStr"/>
+      <c r="O233" t="inlineStr"/>
+      <c r="P233" t="inlineStr"/>
+      <c r="Q233" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:28:01</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr"/>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J234" t="n">
+        <v>1.8791</v>
+      </c>
+      <c r="K234" t="n">
+        <v>8.08</v>
+      </c>
+      <c r="L234" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>Soccabet, Sportybet, 22Bet</t>
+        </is>
+      </c>
+      <c r="N234" t="inlineStr"/>
+      <c r="O234" t="inlineStr"/>
+      <c r="P234" t="inlineStr"/>
+      <c r="Q234" t="inlineStr"/>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:28:01</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr"/>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J235" t="n">
+        <v>1.1907</v>
+      </c>
+      <c r="K235" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="L235" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>Soccabet, 22Bet, Sportybet</t>
+        </is>
+      </c>
+      <c r="N235" t="inlineStr"/>
+      <c r="O235" t="inlineStr"/>
+      <c r="P235" t="inlineStr"/>
+      <c r="Q235" t="inlineStr"/>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:30:51</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr"/>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J236" t="n">
+        <v>1.8791</v>
+      </c>
+      <c r="K236" t="n">
+        <v>8.08</v>
+      </c>
+      <c r="L236" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="M236" t="inlineStr">
+        <is>
+          <t>Soccabet, Sportybet, 22Bet</t>
+        </is>
+      </c>
+      <c r="N236" t="inlineStr"/>
+      <c r="O236" t="inlineStr"/>
+      <c r="P236" t="inlineStr"/>
+      <c r="Q236" t="inlineStr"/>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:30:51</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr"/>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J237" t="n">
+        <v>1.1907</v>
+      </c>
+      <c r="K237" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="L237" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>Soccabet, 22Bet, Sportybet</t>
+        </is>
+      </c>
+      <c r="N237" t="inlineStr"/>
+      <c r="O237" t="inlineStr"/>
+      <c r="P237" t="inlineStr"/>
+      <c r="Q237" t="inlineStr"/>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:33:22</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr"/>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J238" t="n">
+        <v>1.8791</v>
+      </c>
+      <c r="K238" t="n">
+        <v>8.08</v>
+      </c>
+      <c r="L238" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="M238" t="inlineStr">
+        <is>
+          <t>Soccabet, Sportybet, 22Bet</t>
+        </is>
+      </c>
+      <c r="N238" t="inlineStr"/>
+      <c r="O238" t="inlineStr"/>
+      <c r="P238" t="inlineStr"/>
+      <c r="Q238" t="inlineStr"/>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:33:22</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr"/>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J239" t="n">
+        <v>1.1907</v>
+      </c>
+      <c r="K239" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="L239" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>Soccabet, 22Bet, Sportybet</t>
+        </is>
+      </c>
+      <c r="N239" t="inlineStr"/>
+      <c r="O239" t="inlineStr"/>
+      <c r="P239" t="inlineStr"/>
+      <c r="Q239" t="inlineStr"/>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:35:45</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr"/>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J240" t="n">
+        <v>1.8791</v>
+      </c>
+      <c r="K240" t="n">
+        <v>8.08</v>
+      </c>
+      <c r="L240" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>Soccabet, Sportybet, 22Bet</t>
+        </is>
+      </c>
+      <c r="N240" t="inlineStr"/>
+      <c r="O240" t="inlineStr"/>
+      <c r="P240" t="inlineStr"/>
+      <c r="Q240" t="inlineStr"/>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:35:45</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr"/>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J241" t="n">
+        <v>1.1907</v>
+      </c>
+      <c r="K241" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="L241" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>Soccabet, 22Bet, Sportybet</t>
+        </is>
+      </c>
+      <c r="N241" t="inlineStr"/>
+      <c r="O241" t="inlineStr"/>
+      <c r="P241" t="inlineStr"/>
+      <c r="Q241" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:38:12</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr"/>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J242" t="n">
+        <v>1.8791</v>
+      </c>
+      <c r="K242" t="n">
+        <v>8.08</v>
+      </c>
+      <c r="L242" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>Soccabet, Sportybet, 22Bet</t>
+        </is>
+      </c>
+      <c r="N242" t="inlineStr"/>
+      <c r="O242" t="inlineStr"/>
+      <c r="P242" t="inlineStr"/>
+      <c r="Q242" t="inlineStr"/>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-06-18 17:38:12</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr"/>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J243" t="n">
+        <v>1.1907</v>
+      </c>
+      <c r="K243" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="L243" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>Soccabet, 22Bet, Sportybet</t>
+        </is>
+      </c>
+      <c r="N243" t="inlineStr"/>
+      <c r="O243" t="inlineStr"/>
+      <c r="P243" t="inlineStr"/>
+      <c r="Q243" t="inlineStr"/>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:03:06</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr"/>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="J244" t="n">
+        <v>0.2419</v>
+      </c>
+      <c r="K244" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="L244" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>1xBet, Sportybet, Soccabet</t>
+        </is>
+      </c>
+      <c r="N244" t="inlineStr"/>
+      <c r="O244" t="inlineStr"/>
+      <c r="P244" t="inlineStr"/>
+      <c r="Q244" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:03:06</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr"/>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="J245" t="n">
+        <v>1.7209</v>
+      </c>
+      <c r="K245" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="L245" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="M245" t="inlineStr">
+        <is>
+          <t>1xBet, Soccabet, Soccabet</t>
+        </is>
+      </c>
+      <c r="N245" t="inlineStr"/>
+      <c r="O245" t="inlineStr"/>
+      <c r="P245" t="inlineStr"/>
+      <c r="Q245" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:03:06</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr"/>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="J246" t="n">
+        <v>1.7535</v>
+      </c>
+      <c r="K246" t="n">
+        <v>7.54</v>
+      </c>
+      <c r="L246" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>Soccabet, Sportybet, Sportybet</t>
+        </is>
+      </c>
+      <c r="N246" t="inlineStr"/>
+      <c r="O246" t="inlineStr"/>
+      <c r="P246" t="inlineStr"/>
+      <c r="Q246" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:03:06</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr"/>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="J247" t="n">
+        <v>1.6279</v>
+      </c>
+      <c r="K247" t="n">
+        <v>7</v>
+      </c>
+      <c r="L247" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>Soccabet, Sportybet, 1xBet</t>
+        </is>
+      </c>
+      <c r="N247" t="inlineStr"/>
+      <c r="O247" t="inlineStr"/>
+      <c r="P247" t="inlineStr"/>
+      <c r="Q247" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:03:06</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr"/>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J248" t="n">
+        <v>1.8791</v>
+      </c>
+      <c r="K248" t="n">
+        <v>8.08</v>
+      </c>
+      <c r="L248" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>Soccabet, Sportybet, 22Bet</t>
+        </is>
+      </c>
+      <c r="N248" t="inlineStr"/>
+      <c r="O248" t="inlineStr"/>
+      <c r="P248" t="inlineStr"/>
+      <c r="Q248" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:03:06</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr"/>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J249" t="n">
+        <v>1.1907</v>
+      </c>
+      <c r="K249" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="L249" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M249" t="inlineStr">
+        <is>
+          <t>Soccabet, 22Bet, Sportybet</t>
+        </is>
+      </c>
+      <c r="N249" t="inlineStr"/>
+      <c r="O249" t="inlineStr"/>
+      <c r="P249" t="inlineStr"/>
+      <c r="Q249" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:03:06</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr"/>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="J250" t="n">
+        <v>1.0651</v>
+      </c>
+      <c r="K250" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="L250" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M250" t="inlineStr">
+        <is>
+          <t>Soccabet, 22Bet, 1xBet</t>
+        </is>
+      </c>
+      <c r="N250" t="inlineStr"/>
+      <c r="O250" t="inlineStr"/>
+      <c r="P250" t="inlineStr"/>
+      <c r="Q250" t="inlineStr"/>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:03:06</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr"/>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J251" t="n">
+        <v>1.3209</v>
+      </c>
+      <c r="K251" t="n">
+        <v>5.68</v>
+      </c>
+      <c r="L251" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>Soccabet, 22Bet, 22Bet</t>
+        </is>
+      </c>
+      <c r="N251" t="inlineStr"/>
+      <c r="O251" t="inlineStr"/>
+      <c r="P251" t="inlineStr"/>
+      <c r="Q251" t="inlineStr"/>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:05:39</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr"/>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="J252" t="n">
+        <v>1.3465</v>
+      </c>
+      <c r="K252" t="n">
+        <v>5.79</v>
+      </c>
+      <c r="L252" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>Soccabet, Sportybet, 1xBet</t>
+        </is>
+      </c>
+      <c r="N252" t="inlineStr"/>
+      <c r="O252" t="inlineStr"/>
+      <c r="P252" t="inlineStr"/>
+      <c r="Q252" t="inlineStr"/>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:05:39</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr"/>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J253" t="n">
+        <v>0.2953</v>
+      </c>
+      <c r="K253" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="L253" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>Soccabet, Sportybet, 22Bet</t>
+        </is>
+      </c>
+      <c r="N253" t="inlineStr"/>
+      <c r="O253" t="inlineStr"/>
+      <c r="P253" t="inlineStr"/>
+      <c r="Q253" t="inlineStr"/>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:09:05</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr"/>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="J254" t="n">
+        <v>0.2419</v>
+      </c>
+      <c r="K254" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="L254" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="M254" t="inlineStr">
+        <is>
+          <t>1xBet, Sportybet, Soccabet</t>
+        </is>
+      </c>
+      <c r="N254" t="inlineStr"/>
+      <c r="O254" t="inlineStr"/>
+      <c r="P254" t="inlineStr"/>
+      <c r="Q254" t="inlineStr"/>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:09:05</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr"/>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="J255" t="n">
+        <v>1.7209</v>
+      </c>
+      <c r="K255" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="L255" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="M255" t="inlineStr">
+        <is>
+          <t>1xBet, Soccabet, Soccabet</t>
+        </is>
+      </c>
+      <c r="N255" t="inlineStr"/>
+      <c r="O255" t="inlineStr"/>
+      <c r="P255" t="inlineStr"/>
+      <c r="Q255" t="inlineStr"/>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:09:05</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr"/>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="J256" t="n">
+        <v>1.3465</v>
+      </c>
+      <c r="K256" t="n">
+        <v>5.79</v>
+      </c>
+      <c r="L256" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>Soccabet, Sportybet, 1xBet</t>
+        </is>
+      </c>
+      <c r="N256" t="inlineStr"/>
+      <c r="O256" t="inlineStr"/>
+      <c r="P256" t="inlineStr"/>
+      <c r="Q256" t="inlineStr"/>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:09:05</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr"/>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="J257" t="n">
+        <v>0.2953</v>
+      </c>
+      <c r="K257" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="L257" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>Soccabet, Sportybet, 22Bet</t>
+        </is>
+      </c>
+      <c r="N257" t="inlineStr"/>
+      <c r="O257" t="inlineStr"/>
+      <c r="P257" t="inlineStr"/>
+      <c r="Q257" t="inlineStr"/>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-06-18 18:09:05</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Bosnia &amp; Herzegovina</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>World Cup</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr"/>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="J258" t="n">
+        <v>1.0651</v>
+      </c>
+      <c r="K258" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="L258" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>Soccabet, 22Bet, 1xBet</t>
+        </is>
+      </c>
+      <c r="N258" t="inlineStr"/>
+      <c r="O258" t="inlineStr"/>
+      <c r="P258" t="inlineStr"/>
+      <c r="Q258" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>